<commit_message>
FU******* LOTS OF UPDATEES ARGHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHHH
</commit_message>
<xml_diff>
--- a/dist/data/events.xlsx
+++ b/dist/data/events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Codes\r-shs\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA216346-0BBB-46A6-A3C8-82597BAE36C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DEB5D6-EE95-4B49-A80C-970ED213EB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9645" yWindow="5670" windowWidth="20385" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="4515" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>name</t>
   </si>
@@ -54,19 +54,7 @@
     <t>/r-shs/</t>
   </si>
   <si>
-    <t>Jingle Joyce</t>
-  </si>
-  <si>
     <t>Events</t>
-  </si>
-  <si>
-    <t>/r-shs/Christmas</t>
-  </si>
-  <si>
-    <t>Slither Sweetheart</t>
-  </si>
-  <si>
-    <t>/r-shs/Valentine</t>
   </si>
   <si>
     <t>Recup</t>
@@ -396,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="28.140625" customWidth="1"/>
@@ -429,46 +417,24 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>